<commit_message>
Updated description, message and output variables as requested in the PR.
</commit_message>
<xml_diff>
--- a/rules/CORE-000140/negative/01/data/unit-test-coreid-CG0225-negative 1.xlsx
+++ b/rules/CORE-000140/negative/01/data/unit-test-coreid-CG0225-negative 1.xlsx
@@ -37,7 +37,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x14ac">
   <numFmts count="0"/>
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
@@ -54,6 +54,10 @@
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
       <i/>
     </font>
     <font>
@@ -65,7 +69,7 @@
       <name val="Calibri"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none">
         <bgColor/>
@@ -79,6 +83,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FFFFCC"/>
+        <bgColor/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
         <bgColor/>
       </patternFill>
     </fill>
@@ -108,14 +118,15 @@
   <cellStyleXfs>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="1" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -458,10 +469,10 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="str">
+      <c r="A2" s="4" t="str">
         <v>sdtmig</v>
       </c>
-      <c r="B2" s="2" t="str">
+      <c r="B2" s="4" t="str">
         <v>3-4</v>
       </c>
     </row>
@@ -485,18 +496,18 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="str">
+      <c r="A2" s="4" t="str">
         <v>tv.xpt</v>
       </c>
-      <c r="B2" s="2" t="str">
+      <c r="B2" s="4" t="str">
         <v>Trial Visits</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="str">
+      <c r="A3" s="4" t="str">
         <v>sv.xpt</v>
       </c>
-      <c r="B3" s="2" t="str">
+      <c r="B3" s="4" t="str">
         <v>Subject Visits</v>
       </c>
     </row>
@@ -509,7 +520,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F4"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="3" t="str">
@@ -532,48 +543,68 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2">
+      <c r="A2" s="4">
         <v>1</v>
       </c>
-      <c r="B2" s="2" t="str">
+      <c r="B2" s="4" t="str">
         <v>sv.xpt</v>
       </c>
-      <c r="C2" s="2" t="str">
+      <c r="C2" s="4" t="str">
         <v>Record</v>
       </c>
-      <c r="D2" s="2">
+      <c r="D2" s="4">
         <v>10</v>
       </c>
-      <c r="E2" s="2" t="str">
+      <c r="E2" s="4" t="str">
+        <v>VISIT</v>
+      </c>
+      <c r="F2" s="4" t="str">
+        <v>WEEK 4: UNSCHEDULED 01</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4">
+        <v>1</v>
+      </c>
+      <c r="B3" s="4" t="str">
+        <v>sv.xpt</v>
+      </c>
+      <c r="C3" s="4" t="str">
+        <v>Record</v>
+      </c>
+      <c r="D3" s="4">
+        <v>10</v>
+      </c>
+      <c r="E3" s="4" t="str">
         <v>VISITDY</v>
       </c>
-      <c r="F2" s="2">
+      <c r="F3" s="4">
         <v>40</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="2">
+    <row r="4">
+      <c r="A4" s="4">
         <v>1</v>
       </c>
-      <c r="B3" s="2" t="str">
+      <c r="B4" s="4" t="str">
         <v>sv.xpt</v>
       </c>
-      <c r="C3" s="2" t="str">
+      <c r="C4" s="4" t="str">
         <v>Record</v>
       </c>
-      <c r="D3" s="2">
+      <c r="D4" s="4">
         <v>10</v>
       </c>
-      <c r="E3" s="2" t="str">
+      <c r="E4" s="4" t="str">
         <v>VISITNUM</v>
       </c>
-      <c r="F3" s="2">
+      <c r="F4" s="4">
         <v>5.01</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F4"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -609,405 +640,405 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="4" t="str">
+      <c r="A2" s="5" t="str">
         <v>Study Identifier</v>
       </c>
-      <c r="B2" s="4" t="str">
+      <c r="B2" s="5" t="str">
         <v>Domain Abbreviation</v>
       </c>
-      <c r="C2" s="4" t="str">
+      <c r="C2" s="5" t="str">
         <v>Visit Number</v>
       </c>
-      <c r="D2" s="4" t="str">
+      <c r="D2" s="5" t="str">
         <v>Visit Name</v>
       </c>
-      <c r="E2" s="4" t="str">
+      <c r="E2" s="5" t="str">
         <v>Planned Study Day of Visit</v>
       </c>
-      <c r="F2" s="4" t="str">
+      <c r="F2" s="5" t="str">
         <v>Planned Arm Code</v>
       </c>
-      <c r="G2" s="4" t="str">
+      <c r="G2" s="5" t="str">
         <v>Visit Start Rule</v>
       </c>
-      <c r="H2" s="4" t="str">
+      <c r="H2" s="5" t="str">
         <v>Visit End Rule</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="4" t="str">
+      <c r="A3" s="5" t="str">
         <v>Char</v>
       </c>
-      <c r="B3" s="4" t="str">
+      <c r="B3" s="5" t="str">
         <v>Char</v>
       </c>
-      <c r="C3" s="4" t="str">
+      <c r="C3" s="5" t="str">
         <v>Num</v>
       </c>
-      <c r="D3" s="4" t="str">
+      <c r="D3" s="5" t="str">
         <v>Char</v>
       </c>
-      <c r="E3" s="4" t="str">
+      <c r="E3" s="5" t="str">
         <v>Num</v>
       </c>
-      <c r="F3" s="4" t="str">
+      <c r="F3" s="5" t="str">
         <v>Char</v>
       </c>
-      <c r="G3" s="4" t="str">
+      <c r="G3" s="5" t="str">
         <v>Char</v>
       </c>
-      <c r="H3" s="4" t="str">
+      <c r="H3" s="5" t="str">
         <v>Char</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4">
+      <c r="A4" s="5">
         <v>12</v>
       </c>
-      <c r="B4" s="4">
+      <c r="B4" s="5">
         <v>2</v>
       </c>
-      <c r="C4" s="4">
+      <c r="C4" s="5">
         <v>8</v>
       </c>
-      <c r="D4" s="4">
+      <c r="D4" s="5">
         <v>200</v>
       </c>
-      <c r="E4" s="4">
+      <c r="E4" s="5">
         <v>8</v>
       </c>
-      <c r="F4" s="4">
+      <c r="F4" s="5">
         <v>8</v>
       </c>
-      <c r="G4" s="4">
+      <c r="G4" s="5">
         <v>200</v>
       </c>
-      <c r="H4" s="4">
+      <c r="H4" s="5">
         <v>200</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="5" t="str">
-        <v>CDISCPILOT01</v>
-      </c>
-      <c r="B5" s="5" t="str">
+      <c r="A5" s="4" t="str">
+        <v>CDISCPILOT01</v>
+      </c>
+      <c r="B5" s="4" t="str">
         <v>TV</v>
       </c>
-      <c r="C5" s="5">
+      <c r="C5" s="4">
         <v>1</v>
       </c>
-      <c r="D5" s="5" t="str">
+      <c r="D5" s="4" t="str">
         <v>SCREENING 1</v>
       </c>
-      <c r="E5" s="2" t="str">
-        <v/>
-      </c>
-      <c r="F5" s="2" t="str">
-        <v/>
-      </c>
-      <c r="G5" s="5" t="str">
+      <c r="E5" s="4" t="str">
+        <v/>
+      </c>
+      <c r="F5" s="4" t="str">
+        <v/>
+      </c>
+      <c r="G5" s="4" t="str">
         <v>Informed Consent Obtained</v>
       </c>
-      <c r="H5" s="5" t="str">
+      <c r="H5" s="4" t="str">
         <v>Screening Assessments Completed</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="5" t="str">
-        <v>CDISCPILOT01</v>
-      </c>
-      <c r="B6" s="5" t="str">
+      <c r="A6" s="4" t="str">
+        <v>CDISCPILOT01</v>
+      </c>
+      <c r="B6" s="4" t="str">
         <v>TV</v>
       </c>
-      <c r="C6" s="5">
+      <c r="C6" s="4">
         <v>2</v>
       </c>
-      <c r="D6" s="5" t="str">
+      <c r="D6" s="4" t="str">
         <v>SCREENING 2</v>
       </c>
-      <c r="E6" s="2" t="str">
-        <v/>
-      </c>
-      <c r="F6" s="2" t="str">
-        <v/>
-      </c>
-      <c r="G6" s="5" t="str">
+      <c r="E6" s="4" t="str">
+        <v/>
+      </c>
+      <c r="F6" s="4" t="str">
+        <v/>
+      </c>
+      <c r="G6" s="4" t="str">
         <v>Day Before Initial Study Treatment</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="5" t="str">
-        <v>CDISCPILOT01</v>
-      </c>
-      <c r="B7" s="5" t="str">
+      <c r="A7" s="4" t="str">
+        <v>CDISCPILOT01</v>
+      </c>
+      <c r="B7" s="4" t="str">
         <v>TV</v>
       </c>
-      <c r="C7" s="5">
+      <c r="C7" s="4">
         <v>3</v>
       </c>
-      <c r="D7" s="5" t="str">
+      <c r="D7" s="4" t="str">
         <v>BASELINE</v>
       </c>
-      <c r="E7" s="2" t="str">
-        <v/>
-      </c>
-      <c r="F7" s="2" t="str">
-        <v/>
-      </c>
-      <c r="G7" s="5" t="str">
+      <c r="E7" s="4" t="str">
+        <v/>
+      </c>
+      <c r="F7" s="4" t="str">
+        <v/>
+      </c>
+      <c r="G7" s="4" t="str">
         <v>Day of Initial Study Treatment</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="5" t="str">
-        <v>CDISCPILOT01</v>
-      </c>
-      <c r="B8" s="5" t="str">
+      <c r="A8" s="4" t="str">
+        <v>CDISCPILOT01</v>
+      </c>
+      <c r="B8" s="4" t="str">
         <v>TV</v>
       </c>
-      <c r="C8" s="5">
+      <c r="C8" s="4">
         <v>4</v>
       </c>
-      <c r="D8" s="5" t="str">
+      <c r="D8" s="4" t="str">
         <v>WEEK 2</v>
       </c>
-      <c r="E8" s="2" t="str">
-        <v/>
-      </c>
-      <c r="F8" s="2" t="str">
-        <v/>
-      </c>
-      <c r="G8" s="5" t="str">
+      <c r="E8" s="4" t="str">
+        <v/>
+      </c>
+      <c r="F8" s="4" t="str">
+        <v/>
+      </c>
+      <c r="G8" s="4" t="str">
         <v>2 Weeks After Start of Study Treatment</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="5" t="str">
-        <v>CDISCPILOT01</v>
-      </c>
-      <c r="B9" s="5" t="str">
+      <c r="A9" s="4" t="str">
+        <v>CDISCPILOT01</v>
+      </c>
+      <c r="B9" s="4" t="str">
         <v>TV</v>
       </c>
-      <c r="C9" s="5">
+      <c r="C9" s="4">
         <v>5</v>
       </c>
-      <c r="D9" s="5" t="str">
+      <c r="D9" s="4" t="str">
         <v>WEEK 4</v>
       </c>
-      <c r="E9" s="2" t="str">
-        <v/>
-      </c>
-      <c r="F9" s="2" t="str">
-        <v/>
-      </c>
-      <c r="G9" s="5" t="str">
+      <c r="E9" s="4" t="str">
+        <v/>
+      </c>
+      <c r="F9" s="4" t="str">
+        <v/>
+      </c>
+      <c r="G9" s="4" t="str">
         <v>4 Weeks After Start of Study Treatment</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="5" t="str">
-        <v>CDISCPILOT01</v>
-      </c>
-      <c r="B10" s="5" t="str">
+      <c r="A10" s="4" t="str">
+        <v>CDISCPILOT01</v>
+      </c>
+      <c r="B10" s="4" t="str">
         <v>TV</v>
       </c>
-      <c r="C10" s="5">
+      <c r="C10" s="4">
         <v>7</v>
       </c>
-      <c r="D10" s="5" t="str">
+      <c r="D10" s="4" t="str">
         <v>WEEK 6</v>
       </c>
-      <c r="E10" s="2" t="str">
-        <v/>
-      </c>
-      <c r="F10" s="2" t="str">
-        <v/>
-      </c>
-      <c r="G10" s="5" t="str">
+      <c r="E10" s="4" t="str">
+        <v/>
+      </c>
+      <c r="F10" s="4" t="str">
+        <v/>
+      </c>
+      <c r="G10" s="4" t="str">
         <v>6 Weeks After Start of Study Treatment</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="5" t="str">
-        <v>CDISCPILOT01</v>
-      </c>
-      <c r="B11" s="5" t="str">
+      <c r="A11" s="4" t="str">
+        <v>CDISCPILOT01</v>
+      </c>
+      <c r="B11" s="4" t="str">
         <v>TV</v>
       </c>
-      <c r="C11" s="5">
+      <c r="C11" s="4">
         <v>8</v>
       </c>
-      <c r="D11" s="5" t="str">
+      <c r="D11" s="4" t="str">
         <v>WEEK 8</v>
       </c>
-      <c r="E11" s="2" t="str">
-        <v/>
-      </c>
-      <c r="F11" s="2" t="str">
-        <v/>
-      </c>
-      <c r="G11" s="5" t="str">
+      <c r="E11" s="4" t="str">
+        <v/>
+      </c>
+      <c r="F11" s="4" t="str">
+        <v/>
+      </c>
+      <c r="G11" s="4" t="str">
         <v>8 Weeks After Start of Study Treatment</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="5" t="str">
-        <v>CDISCPILOT01</v>
-      </c>
-      <c r="B12" s="5" t="str">
+      <c r="A12" s="4" t="str">
+        <v>CDISCPILOT01</v>
+      </c>
+      <c r="B12" s="4" t="str">
         <v>TV</v>
       </c>
-      <c r="C12" s="5">
+      <c r="C12" s="4">
         <v>9</v>
       </c>
-      <c r="D12" s="5" t="str">
+      <c r="D12" s="4" t="str">
         <v>WEEK 12</v>
       </c>
-      <c r="E12" s="2" t="str">
-        <v/>
-      </c>
-      <c r="F12" s="2" t="str">
-        <v/>
-      </c>
-      <c r="G12" s="5" t="str">
+      <c r="E12" s="4" t="str">
+        <v/>
+      </c>
+      <c r="F12" s="4" t="str">
+        <v/>
+      </c>
+      <c r="G12" s="4" t="str">
         <v>12 Weeks After Start of Study Treatment</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="5" t="str">
-        <v>CDISCPILOT01</v>
-      </c>
-      <c r="B13" s="5" t="str">
+      <c r="A13" s="4" t="str">
+        <v>CDISCPILOT01</v>
+      </c>
+      <c r="B13" s="4" t="str">
         <v>TV</v>
       </c>
-      <c r="C13" s="5">
+      <c r="C13" s="4">
         <v>10</v>
       </c>
-      <c r="D13" s="5" t="str">
+      <c r="D13" s="4" t="str">
         <v>WEEK 16</v>
       </c>
-      <c r="E13" s="2" t="str">
-        <v/>
-      </c>
-      <c r="F13" s="2" t="str">
-        <v/>
-      </c>
-      <c r="G13" s="5" t="str">
+      <c r="E13" s="4" t="str">
+        <v/>
+      </c>
+      <c r="F13" s="4" t="str">
+        <v/>
+      </c>
+      <c r="G13" s="4" t="str">
         <v>16 Weeks After Start of Study Treatment</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="5" t="str">
-        <v>CDISCPILOT01</v>
-      </c>
-      <c r="B14" s="5" t="str">
+      <c r="A14" s="4" t="str">
+        <v>CDISCPILOT01</v>
+      </c>
+      <c r="B14" s="4" t="str">
         <v>TV</v>
       </c>
-      <c r="C14" s="5">
+      <c r="C14" s="4">
         <v>11</v>
       </c>
-      <c r="D14" s="5" t="str">
+      <c r="D14" s="4" t="str">
         <v>WEEK 20</v>
       </c>
-      <c r="E14" s="2" t="str">
-        <v/>
-      </c>
-      <c r="F14" s="2" t="str">
-        <v/>
-      </c>
-      <c r="G14" s="5" t="str">
+      <c r="E14" s="4" t="str">
+        <v/>
+      </c>
+      <c r="F14" s="4" t="str">
+        <v/>
+      </c>
+      <c r="G14" s="4" t="str">
         <v>20 Weeks After Start of Study Treatment</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="5" t="str">
-        <v>CDISCPILOT01</v>
-      </c>
-      <c r="B15" s="5" t="str">
+      <c r="A15" s="4" t="str">
+        <v>CDISCPILOT01</v>
+      </c>
+      <c r="B15" s="4" t="str">
         <v>TV</v>
       </c>
-      <c r="C15" s="5">
+      <c r="C15" s="4">
         <v>12</v>
       </c>
-      <c r="D15" s="5" t="str">
+      <c r="D15" s="4" t="str">
         <v>WEEK 24</v>
       </c>
-      <c r="E15" s="2" t="str">
-        <v/>
-      </c>
-      <c r="F15" s="2" t="str">
-        <v/>
-      </c>
-      <c r="G15" s="5" t="str">
+      <c r="E15" s="4" t="str">
+        <v/>
+      </c>
+      <c r="F15" s="4" t="str">
+        <v/>
+      </c>
+      <c r="G15" s="4" t="str">
         <v>24 Weeks After Start of Study Treatment</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="5" t="str">
-        <v>CDISCPILOT01</v>
-      </c>
-      <c r="B16" s="5" t="str">
+      <c r="A16" s="4" t="str">
+        <v>CDISCPILOT01</v>
+      </c>
+      <c r="B16" s="4" t="str">
         <v>TV</v>
       </c>
-      <c r="C16" s="5">
+      <c r="C16" s="4">
         <v>13</v>
       </c>
-      <c r="D16" s="5" t="str">
+      <c r="D16" s="4" t="str">
         <v>WEEK 26</v>
       </c>
-      <c r="E16" s="2" t="str">
-        <v/>
-      </c>
-      <c r="F16" s="2" t="str">
-        <v/>
-      </c>
-      <c r="G16" s="5" t="str">
+      <c r="E16" s="4" t="str">
+        <v/>
+      </c>
+      <c r="F16" s="4" t="str">
+        <v/>
+      </c>
+      <c r="G16" s="4" t="str">
         <v>26 Weeks After Start of Study Treatment</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="5" t="str">
-        <v>CDISCPILOT01</v>
-      </c>
-      <c r="B17" s="5" t="str">
+      <c r="A17" s="4" t="str">
+        <v>CDISCPILOT01</v>
+      </c>
+      <c r="B17" s="4" t="str">
         <v>TV</v>
       </c>
-      <c r="C17" s="5">
+      <c r="C17" s="4">
         <v>101</v>
       </c>
-      <c r="D17" s="5" t="str">
+      <c r="D17" s="4" t="str">
         <v>EARLY DISCONTINUATION</v>
       </c>
-      <c r="E17" s="2" t="str">
-        <v/>
-      </c>
-      <c r="F17" s="2" t="str">
-        <v/>
-      </c>
-      <c r="G17" s="5" t="str">
+      <c r="E17" s="4" t="str">
+        <v/>
+      </c>
+      <c r="F17" s="4" t="str">
+        <v/>
+      </c>
+      <c r="G17" s="4" t="str">
         <v>Discontinuation Date Prior to Week 24</v>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="5" t="str">
-        <v>CDISCPILOT01</v>
-      </c>
-      <c r="B18" s="5" t="str">
+      <c r="A18" s="4" t="str">
+        <v>CDISCPILOT01</v>
+      </c>
+      <c r="B18" s="4" t="str">
         <v>TV</v>
       </c>
-      <c r="C18" s="5">
+      <c r="C18" s="4">
         <v>201</v>
       </c>
-      <c r="D18" s="5" t="str">
+      <c r="D18" s="4" t="str">
         <v>EARLY DISCONTINUATION RETRIEVAL</v>
       </c>
-      <c r="E18" s="2" t="str">
-        <v/>
-      </c>
-      <c r="F18" s="2" t="str">
-        <v/>
-      </c>
-      <c r="G18" s="5" t="str">
+      <c r="E18" s="4" t="str">
+        <v/>
+      </c>
+      <c r="F18" s="4" t="str">
+        <v/>
+      </c>
+      <c r="G18" s="4" t="str">
         <v>Approximately 24 Weeks After Start of Study Treatment for Early Discontinuations</v>
       </c>
     </row>
@@ -1058,302 +1089,302 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="4" t="str">
+      <c r="A2" s="5" t="str">
         <v>Study Identifier</v>
       </c>
-      <c r="B2" s="4" t="str">
+      <c r="B2" s="5" t="str">
         <v>Domain Abbreviation</v>
       </c>
-      <c r="C2" s="4" t="str">
+      <c r="C2" s="5" t="str">
         <v>Unique Subject Identifier</v>
       </c>
-      <c r="D2" s="4" t="str">
+      <c r="D2" s="5" t="str">
         <v>Visit Number</v>
       </c>
-      <c r="E2" s="4" t="str">
+      <c r="E2" s="5" t="str">
         <v>Visit Name</v>
       </c>
-      <c r="F2" s="4" t="str">
+      <c r="F2" s="5" t="str">
         <v>Planned Study Day of Visit</v>
       </c>
-      <c r="G2" s="4" t="str">
+      <c r="G2" s="5" t="str">
         <v>Start Date/Time of Visit</v>
       </c>
-      <c r="H2" s="4" t="str">
+      <c r="H2" s="5" t="str">
         <v>End Date/Time of Visit</v>
       </c>
-      <c r="I2" s="4" t="str">
+      <c r="I2" s="5" t="str">
         <v>Study Day of Start of Visit</v>
       </c>
-      <c r="J2" s="4" t="str">
+      <c r="J2" s="5" t="str">
         <v>Study Day of End of Visit</v>
       </c>
-      <c r="K2" s="4" t="str">
+      <c r="K2" s="5" t="str">
         <v>Description of Unplanned Visit</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="4" t="str">
+      <c r="A3" s="5" t="str">
         <v>Char</v>
       </c>
-      <c r="B3" s="4" t="str">
+      <c r="B3" s="5" t="str">
         <v>Char</v>
       </c>
-      <c r="C3" s="4" t="str">
+      <c r="C3" s="5" t="str">
         <v>Char</v>
       </c>
-      <c r="D3" s="4" t="str">
+      <c r="D3" s="5" t="str">
         <v>Num</v>
       </c>
-      <c r="E3" s="4" t="str">
+      <c r="E3" s="5" t="str">
         <v>Char</v>
       </c>
-      <c r="F3" s="4" t="str">
+      <c r="F3" s="5" t="str">
         <v>Num</v>
       </c>
-      <c r="G3" s="4" t="str">
+      <c r="G3" s="5" t="str">
         <v>Char</v>
       </c>
-      <c r="H3" s="4" t="str">
+      <c r="H3" s="5" t="str">
         <v>Char</v>
       </c>
-      <c r="I3" s="4" t="str">
+      <c r="I3" s="5" t="str">
         <v>Num</v>
       </c>
-      <c r="J3" s="4" t="str">
+      <c r="J3" s="5" t="str">
         <v>Num</v>
       </c>
-      <c r="K3" s="4" t="str">
+      <c r="K3" s="5" t="str">
         <v>Char</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4">
+      <c r="A4" s="5">
         <v>12</v>
       </c>
-      <c r="B4" s="4">
+      <c r="B4" s="5">
         <v>2</v>
       </c>
-      <c r="C4" s="4">
+      <c r="C4" s="5">
         <v>8</v>
       </c>
-      <c r="D4" s="4">
+      <c r="D4" s="5">
         <v>8</v>
       </c>
-      <c r="E4" s="4">
+      <c r="E4" s="5">
         <v>200</v>
       </c>
-      <c r="F4" s="4">
+      <c r="F4" s="5">
         <v>8</v>
       </c>
-      <c r="G4" s="4">
+      <c r="G4" s="5">
         <v>10</v>
       </c>
-      <c r="H4" s="4">
+      <c r="H4" s="5">
         <v>10</v>
       </c>
-      <c r="I4" s="4">
+      <c r="I4" s="5">
         <v>8</v>
       </c>
-      <c r="J4" s="4">
+      <c r="J4" s="5">
         <v>8</v>
       </c>
-      <c r="K4" s="4">
+      <c r="K4" s="5">
         <v>200</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="5" t="str">
-        <v>CDISCPILOT01</v>
-      </c>
-      <c r="B5" s="5" t="str">
+      <c r="A5" s="4" t="str">
+        <v>CDISCPILOT01</v>
+      </c>
+      <c r="B5" s="4" t="str">
         <v>SV</v>
       </c>
-      <c r="C5" s="5" t="str">
+      <c r="C5" s="4" t="str">
         <v>CDISC001</v>
       </c>
-      <c r="D5" s="5">
+      <c r="D5" s="4">
         <v>1</v>
       </c>
-      <c r="E5" s="5" t="str">
+      <c r="E5" s="4" t="str">
         <v>SCREENING 1</v>
       </c>
-      <c r="F5" s="5">
+      <c r="F5" s="4">
         <v>1</v>
       </c>
-      <c r="G5" s="5" t="str">
+      <c r="G5" s="4" t="str">
         <v>2012-11-23</v>
       </c>
-      <c r="H5" s="5" t="str">
+      <c r="H5" s="4" t="str">
         <v>2012-11-23</v>
       </c>
-      <c r="I5" s="5">
+      <c r="I5" s="4">
         <v>-7</v>
       </c>
-      <c r="J5" s="5">
+      <c r="J5" s="4">
         <v>-7</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="5" t="str">
-        <v>CDISCPILOT01</v>
-      </c>
-      <c r="B6" s="5" t="str">
+      <c r="A6" s="4" t="str">
+        <v>CDISCPILOT01</v>
+      </c>
+      <c r="B6" s="4" t="str">
         <v>SV</v>
       </c>
-      <c r="C6" s="5" t="str">
+      <c r="C6" s="4" t="str">
         <v>CDISC001</v>
       </c>
-      <c r="D6" s="5">
+      <c r="D6" s="4">
         <v>2</v>
       </c>
-      <c r="E6" s="5" t="str">
+      <c r="E6" s="4" t="str">
         <v>SCREENING 2</v>
       </c>
-      <c r="F6" s="5">
+      <c r="F6" s="4">
         <v>2</v>
       </c>
-      <c r="G6" s="5" t="str">
+      <c r="G6" s="4" t="str">
         <v>2012-11-28</v>
       </c>
-      <c r="H6" s="5" t="str">
+      <c r="H6" s="4" t="str">
         <v>2012-11-28</v>
       </c>
-      <c r="I6" s="5">
+      <c r="I6" s="4">
         <v>-2</v>
       </c>
-      <c r="J6" s="5">
+      <c r="J6" s="4">
         <v>-2</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="5" t="str">
-        <v>CDISCPILOT01</v>
-      </c>
-      <c r="B7" s="5" t="str">
+      <c r="A7" s="4" t="str">
+        <v>CDISCPILOT01</v>
+      </c>
+      <c r="B7" s="4" t="str">
         <v>SV</v>
       </c>
-      <c r="C7" s="5" t="str">
+      <c r="C7" s="4" t="str">
         <v>CDISC001</v>
       </c>
-      <c r="D7" s="5">
+      <c r="D7" s="4">
         <v>3</v>
       </c>
-      <c r="E7" s="5" t="str">
+      <c r="E7" s="4" t="str">
         <v>BASELINE</v>
       </c>
-      <c r="F7" s="5" t="str">
+      <c r="F7" s="4" t="str">
         <v>11</v>
       </c>
-      <c r="G7" s="5" t="str">
+      <c r="G7" s="4" t="str">
         <v>2012-11-30</v>
       </c>
-      <c r="H7" s="5" t="str">
+      <c r="H7" s="4" t="str">
         <v>2012-11-30</v>
       </c>
-      <c r="I7" s="5">
+      <c r="I7" s="4">
         <v>1</v>
       </c>
-      <c r="J7" s="5">
+      <c r="J7" s="4">
         <v>1</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="5" t="str">
-        <v>CDISCPILOT01</v>
-      </c>
-      <c r="B8" s="5" t="str">
+      <c r="A8" s="4" t="str">
+        <v>CDISCPILOT01</v>
+      </c>
+      <c r="B8" s="4" t="str">
         <v>SV</v>
       </c>
-      <c r="C8" s="5" t="str">
+      <c r="C8" s="4" t="str">
         <v>CDISC001</v>
       </c>
-      <c r="D8" s="5">
+      <c r="D8" s="4">
         <v>4</v>
       </c>
-      <c r="E8" s="5" t="str">
+      <c r="E8" s="4" t="str">
         <v>WEEK 2</v>
       </c>
-      <c r="F8" s="5" t="str">
+      <c r="F8" s="4" t="str">
         <v>18</v>
       </c>
-      <c r="G8" s="5" t="str">
+      <c r="G8" s="4" t="str">
         <v>2012-12-13</v>
       </c>
-      <c r="H8" s="5" t="str">
+      <c r="H8" s="4" t="str">
         <v>2012-12-13</v>
       </c>
-      <c r="I8" s="5">
+      <c r="I8" s="4">
         <v>14</v>
       </c>
-      <c r="J8" s="5">
+      <c r="J8" s="4">
         <v>14</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="5" t="str">
-        <v>CDISCPILOT01</v>
-      </c>
-      <c r="B9" s="5" t="str">
+      <c r="A9" s="4" t="str">
+        <v>CDISCPILOT01</v>
+      </c>
+      <c r="B9" s="4" t="str">
         <v>SV</v>
       </c>
-      <c r="C9" s="5" t="str">
+      <c r="C9" s="4" t="str">
         <v>CDISC001</v>
       </c>
-      <c r="D9" s="5">
+      <c r="D9" s="4">
         <v>5</v>
       </c>
-      <c r="E9" s="5" t="str">
+      <c r="E9" s="4" t="str">
         <v>WEEK 4</v>
       </c>
-      <c r="F9" s="5" t="str">
+      <c r="F9" s="4" t="str">
         <v>39</v>
       </c>
-      <c r="G9" s="5" t="str">
+      <c r="G9" s="4" t="str">
         <v>2012-12-26</v>
       </c>
-      <c r="H9" s="5" t="str">
+      <c r="H9" s="4" t="str">
         <v>2012-12-26</v>
       </c>
-      <c r="I9" s="5">
+      <c r="I9" s="4">
         <v>27</v>
       </c>
-      <c r="J9" s="5">
+      <c r="J9" s="4">
         <v>27</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="5" t="str">
-        <v>CDISCPILOT01</v>
-      </c>
-      <c r="B10" s="5" t="str">
+      <c r="A10" s="4" t="str">
+        <v>CDISCPILOT01</v>
+      </c>
+      <c r="B10" s="4" t="str">
         <v>SV</v>
       </c>
-      <c r="C10" s="5" t="str">
+      <c r="C10" s="4" t="str">
         <v>CDISC001</v>
       </c>
       <c r="D10" s="6">
         <v>5.01</v>
       </c>
-      <c r="E10" s="5" t="str">
+      <c r="E10" s="7" t="str">
         <v>WEEK 4: UNSCHEDULED 01</v>
       </c>
       <c r="F10" s="6" t="str">
         <v>40</v>
       </c>
-      <c r="G10" s="5" t="str">
+      <c r="G10" s="4" t="str">
         <v>2012-12-28</v>
       </c>
-      <c r="H10" s="5" t="str">
+      <c r="H10" s="4" t="str">
         <v>2012-12-28</v>
       </c>
-      <c r="I10" s="5">
+      <c r="I10" s="4">
         <v>29</v>
       </c>
-      <c r="J10" s="5">
+      <c r="J10" s="4">
         <v>29</v>
       </c>
-      <c r="K10" s="5" t="str">
+      <c r="K10" s="4" t="str">
         <v>UNSCHEDULED LABS</v>
       </c>
     </row>

</xml_diff>